<commit_message>
docs(forms): cascade RACI corrections into FRM-202 and FRM-209
- FRM-202 Contract Review Checklist: APPROVAL section restructured from
  3 to 4 sign-off blocks — adds a dedicated Production Director block
  so the manufacturing-feasibility verdict (CDR A5, PD=R) is signed,
  alongside Sales/CS, Engineering and QA/Approver. Rev.01 -> Rev.02.
- FRM-209 High-Risk Job Readiness Review: adds check item #9, a
  shop-floor manufacturability review with the CNC Workshop Manager
  (CDR B1, WKM=C). Rev.01 -> Rev.02.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mom/docs/forms/frm-200-purchase/FRM-202_Contract_Review_Checklist.xlsx
+++ b/mom/docs/forms/frm-200-purchase/FRM-202_Contract_Review_Checklist.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM_202" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTS" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="FRM_202" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LISTS" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -827,7 +827,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="252">
+  <borders count="253">
     <border>
       <left/>
       <right/>
@@ -3651,12 +3651,16 @@
         <color rgb="000078D4"/>
       </bottom>
       <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <bottom/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="517">
+  <cellXfs count="518">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -4906,6 +4910,7 @@
     <xf numFmtId="0" fontId="89" fillId="48" borderId="213" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="252" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5179,36 +5184,6 @@
     </comment>
   </commentList>
 </comments>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>161925</colOff>
-      <row>1</row>
-      <rowOff>314325</rowOff>
-    </from>
-    <ext cx="1123950" cy="323850"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5613,7 +5588,7 @@
       <c r="AH3" s="15" t="n"/>
       <c r="AI3" s="293" t="inlineStr">
         <is>
-          <t>Rev.01</t>
+          <t>Rev.02</t>
         </is>
       </c>
       <c r="AJ3" s="14" t="n"/>
@@ -5656,7 +5631,7 @@
       <c r="AH4" s="15" t="n"/>
       <c r="AI4" s="293" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="AJ4" s="14" t="n"/>
@@ -5746,7 +5721,7 @@
       <c r="AN6" s="272" t="n"/>
     </row>
     <row r="7" ht="4" customHeight="1" s="264">
-      <c r="A7" s="469" t="n"/>
+      <c r="A7" s="517" t="n"/>
       <c r="B7" s="26" t="n"/>
       <c r="C7" s="26" t="n"/>
       <c r="D7" s="26" t="n"/>
@@ -5934,7 +5909,7 @@
       <c r="AN10" s="486" t="n"/>
     </row>
     <row r="11" ht="4" customHeight="1" s="264">
-      <c r="A11" s="469" t="n"/>
+      <c r="A11" s="517" t="n"/>
       <c r="B11" s="26" t="n"/>
       <c r="C11" s="26" t="n"/>
       <c r="D11" s="26" t="n"/>
@@ -6772,7 +6747,7 @@
       <c r="AN25" s="486" t="n"/>
     </row>
     <row r="26" ht="4" customHeight="1" s="264">
-      <c r="A26" s="469" t="n"/>
+      <c r="A26" s="517" t="n"/>
       <c r="B26" s="26" t="n"/>
       <c r="C26" s="26" t="n"/>
       <c r="D26" s="26" t="n"/>
@@ -6873,36 +6848,40 @@
       <c r="G28" s="471" t="n"/>
       <c r="H28" s="471" t="n"/>
       <c r="I28" s="471" t="n"/>
-      <c r="J28" s="471" t="n"/>
-      <c r="K28" s="471" t="n"/>
+      <c r="J28" s="472" t="n"/>
+      <c r="K28" s="509" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
       <c r="L28" s="471" t="n"/>
-      <c r="M28" s="472" t="n"/>
-      <c r="N28" s="509" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
+      <c r="M28" s="471" t="n"/>
+      <c r="N28" s="471" t="n"/>
       <c r="O28" s="471" t="n"/>
       <c r="P28" s="471" t="n"/>
       <c r="Q28" s="471" t="n"/>
       <c r="R28" s="471" t="n"/>
       <c r="S28" s="471" t="n"/>
-      <c r="T28" s="471" t="n"/>
-      <c r="U28" s="471" t="n"/>
+      <c r="T28" s="472" t="n"/>
+      <c r="U28" s="509" t="inlineStr">
+        <is>
+          <t>Production Director</t>
+        </is>
+      </c>
       <c r="V28" s="471" t="n"/>
       <c r="W28" s="471" t="n"/>
       <c r="X28" s="471" t="n"/>
       <c r="Y28" s="471" t="n"/>
-      <c r="Z28" s="472" t="n"/>
-      <c r="AA28" s="509" t="inlineStr">
-        <is>
-          <t>QA / Approver</t>
-        </is>
-      </c>
+      <c r="Z28" s="471" t="n"/>
+      <c r="AA28" s="471" t="n"/>
       <c r="AB28" s="471" t="n"/>
       <c r="AC28" s="471" t="n"/>
-      <c r="AD28" s="471" t="n"/>
-      <c r="AE28" s="471" t="n"/>
+      <c r="AD28" s="472" t="n"/>
+      <c r="AE28" s="509" t="inlineStr">
+        <is>
+          <t>QA / Approver</t>
+        </is>
+      </c>
       <c r="AF28" s="471" t="n"/>
       <c r="AG28" s="471" t="n"/>
       <c r="AH28" s="471" t="n"/>
@@ -6927,36 +6906,40 @@
       <c r="G29" s="511" t="n"/>
       <c r="H29" s="511" t="n"/>
       <c r="I29" s="511" t="n"/>
-      <c r="J29" s="511" t="n"/>
-      <c r="K29" s="511" t="n"/>
+      <c r="J29" s="512" t="n"/>
+      <c r="K29" s="510" t="inlineStr">
+        <is>
+          <t>Name  /  Signature  /  Date</t>
+        </is>
+      </c>
       <c r="L29" s="511" t="n"/>
-      <c r="M29" s="512" t="n"/>
-      <c r="N29" s="510" t="inlineStr">
-        <is>
-          <t>Name  /  Signature  /  Date</t>
-        </is>
-      </c>
+      <c r="M29" s="511" t="n"/>
+      <c r="N29" s="511" t="n"/>
       <c r="O29" s="511" t="n"/>
       <c r="P29" s="511" t="n"/>
       <c r="Q29" s="511" t="n"/>
       <c r="R29" s="511" t="n"/>
       <c r="S29" s="511" t="n"/>
-      <c r="T29" s="511" t="n"/>
-      <c r="U29" s="511" t="n"/>
+      <c r="T29" s="512" t="n"/>
+      <c r="U29" s="510" t="inlineStr">
+        <is>
+          <t>Name  /  Signature  /  Date</t>
+        </is>
+      </c>
       <c r="V29" s="511" t="n"/>
       <c r="W29" s="511" t="n"/>
       <c r="X29" s="511" t="n"/>
       <c r="Y29" s="511" t="n"/>
-      <c r="Z29" s="512" t="n"/>
-      <c r="AA29" s="510" t="inlineStr">
-        <is>
-          <t>Name  /  Signature  /  Date</t>
-        </is>
-      </c>
+      <c r="Z29" s="511" t="n"/>
+      <c r="AA29" s="511" t="n"/>
       <c r="AB29" s="511" t="n"/>
       <c r="AC29" s="511" t="n"/>
-      <c r="AD29" s="511" t="n"/>
-      <c r="AE29" s="511" t="n"/>
+      <c r="AD29" s="512" t="n"/>
+      <c r="AE29" s="510" t="inlineStr">
+        <is>
+          <t>Name  /  Signature  /  Date</t>
+        </is>
+      </c>
       <c r="AF29" s="511" t="n"/>
       <c r="AG29" s="511" t="n"/>
       <c r="AH29" s="511" t="n"/>
@@ -6969,10 +6952,12 @@
     </row>
     <row r="30" ht="26" customHeight="1" s="264">
       <c r="A30" s="513" t="n"/>
-      <c r="M30" s="514" t="n"/>
-      <c r="N30" s="513" t="n"/>
-      <c r="Z30" s="514" t="n"/>
-      <c r="AA30" s="513" t="n"/>
+      <c r="J30" s="514" t="n"/>
+      <c r="K30" s="513" t="n"/>
+      <c r="T30" s="514" t="n"/>
+      <c r="U30" s="513" t="n"/>
+      <c r="AD30" s="514" t="n"/>
+      <c r="AE30" s="513" t="n"/>
       <c r="AN30" s="514" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1" s="264">
@@ -6985,28 +6970,28 @@
       <c r="G31" s="481" t="n"/>
       <c r="H31" s="481" t="n"/>
       <c r="I31" s="481" t="n"/>
-      <c r="J31" s="481" t="n"/>
-      <c r="K31" s="481" t="n"/>
+      <c r="J31" s="486" t="n"/>
+      <c r="K31" s="515" t="n"/>
       <c r="L31" s="481" t="n"/>
-      <c r="M31" s="486" t="n"/>
-      <c r="N31" s="515" t="n"/>
+      <c r="M31" s="481" t="n"/>
+      <c r="N31" s="481" t="n"/>
       <c r="O31" s="481" t="n"/>
       <c r="P31" s="481" t="n"/>
       <c r="Q31" s="481" t="n"/>
       <c r="R31" s="481" t="n"/>
       <c r="S31" s="481" t="n"/>
-      <c r="T31" s="481" t="n"/>
-      <c r="U31" s="481" t="n"/>
+      <c r="T31" s="486" t="n"/>
+      <c r="U31" s="515" t="n"/>
       <c r="V31" s="481" t="n"/>
       <c r="W31" s="481" t="n"/>
       <c r="X31" s="481" t="n"/>
       <c r="Y31" s="481" t="n"/>
-      <c r="Z31" s="486" t="n"/>
-      <c r="AA31" s="515" t="n"/>
+      <c r="Z31" s="481" t="n"/>
+      <c r="AA31" s="481" t="n"/>
       <c r="AB31" s="481" t="n"/>
       <c r="AC31" s="481" t="n"/>
-      <c r="AD31" s="481" t="n"/>
-      <c r="AE31" s="481" t="n"/>
+      <c r="AD31" s="486" t="n"/>
+      <c r="AE31" s="515" t="n"/>
       <c r="AF31" s="481" t="n"/>
       <c r="AG31" s="481" t="n"/>
       <c r="AH31" s="481" t="n"/>
@@ -7018,7 +7003,7 @@
       <c r="AN31" s="486" t="n"/>
     </row>
     <row r="32" ht="4" customHeight="1" s="264">
-      <c r="A32" s="469" t="n"/>
+      <c r="A32" s="517" t="n"/>
       <c r="B32" s="26" t="n"/>
       <c r="C32" s="26" t="n"/>
       <c r="D32" s="26" t="n"/>
@@ -7106,7 +7091,8 @@
       <c r="AN33" s="472" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="114">
+  <mergeCells count="116">
+    <mergeCell ref="AE29:AN31"/>
     <mergeCell ref="F23:U23"/>
     <mergeCell ref="A12:AN12"/>
     <mergeCell ref="A15:B15"/>
@@ -7114,8 +7100,8 @@
     <mergeCell ref="F13:U13"/>
     <mergeCell ref="AE6:AH6"/>
     <mergeCell ref="A32:AN32"/>
+    <mergeCell ref="A29:J31"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="AA28:AN28"/>
     <mergeCell ref="V22:AE22"/>
     <mergeCell ref="AF22:AI22"/>
     <mergeCell ref="A9:G9"/>
@@ -7150,7 +7136,6 @@
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="AJ14:AN14"/>
     <mergeCell ref="AE5:AH5"/>
-    <mergeCell ref="A28:M28"/>
     <mergeCell ref="AJ23:AN23"/>
     <mergeCell ref="U10:AA10"/>
     <mergeCell ref="AB10:AN10"/>
@@ -7172,16 +7157,18 @@
     <mergeCell ref="V15:AE15"/>
     <mergeCell ref="AF20:AI20"/>
     <mergeCell ref="AF14:AI14"/>
+    <mergeCell ref="U28:AD28"/>
     <mergeCell ref="A27:AN27"/>
     <mergeCell ref="C16:E16"/>
+    <mergeCell ref="AE28:AN28"/>
     <mergeCell ref="F22:U22"/>
     <mergeCell ref="A33:AN33"/>
-    <mergeCell ref="AA29:AN31"/>
-    <mergeCell ref="N29:Z31"/>
     <mergeCell ref="V16:AE16"/>
+    <mergeCell ref="A28:J28"/>
     <mergeCell ref="AF13:AI13"/>
     <mergeCell ref="F14:U14"/>
     <mergeCell ref="V18:AE18"/>
+    <mergeCell ref="U29:AD31"/>
     <mergeCell ref="AJ13:AN13"/>
     <mergeCell ref="I6:AD6"/>
     <mergeCell ref="A21:B21"/>
@@ -7199,14 +7186,13 @@
     <mergeCell ref="AI6:AN6"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A26:AN26"/>
-    <mergeCell ref="N28:Z28"/>
     <mergeCell ref="AF17:AI17"/>
     <mergeCell ref="AI4:AN4"/>
-    <mergeCell ref="A29:M31"/>
     <mergeCell ref="A8:AN8"/>
     <mergeCell ref="AJ17:AN17"/>
     <mergeCell ref="AF19:AI19"/>
     <mergeCell ref="A16:B16"/>
+    <mergeCell ref="K28:T28"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="AJ19:AN19"/>
@@ -7215,6 +7201,7 @@
     <mergeCell ref="F25:U25"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="AE2:AH2"/>
+    <mergeCell ref="K29:T31"/>
     <mergeCell ref="F15:U15"/>
     <mergeCell ref="V24:AE24"/>
     <mergeCell ref="V19:AE19"/>
@@ -7240,7 +7227,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>

</xml_diff>